<commit_message>
Add chess to chess board
Add chess to chess board
</commit_message>
<xml_diff>
--- a/ConfigExporter/xlsx/game_prefab.xlsx
+++ b/ConfigExporter/xlsx/game_prefab.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Project\WeiqiXN\ConfigExporter\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC2A8EC9-46B7-4FA3-80DE-6EF2F06EA406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61A47FC-5FF3-46ED-BB3C-1FF84E53F1C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8235" yWindow="3270" windowWidth="22170" windowHeight="16605" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8565" yWindow="1170" windowWidth="22170" windowHeight="16605" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="game_prefab" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -88,6 +88,22 @@
   </si>
   <si>
     <t>Models/VFX/FX_LootDrop_Blue</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ChessBlack</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Models/Chess/ChessBlack</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ChessWhite</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Models/Chess/ChessWhite</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -450,7 +466,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.875" style="1" customWidth="1"/>
@@ -533,6 +549,24 @@
         <v>15</v>
       </c>
     </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>